<commit_message>
Add closing period reporting and expand live Excel pivots
</commit_message>
<xml_diff>
--- a/backend/app/services/unaccounted/pivot_templates/pending_mrn_vendorwise.xlsx
+++ b/backend/app/services/unaccounted/pivot_templates/pending_mrn_vendorwise.xlsx
@@ -3,20 +3,21 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="390" yWindow="585" windowWidth="19815" windowHeight="8640" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="390" yWindow="585" windowWidth="19815" windowHeight="8640" tabRatio="600" firstSheet="1" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Locationwise Pivot" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vendorwise Pivot" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_PivotSrc" sheetId="1" state="hidden" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Locationwise Pivot" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vendorwise Pivot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Locationwise Pivot'!$A$1:$D$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Summary'!$A$1:$V$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Summary'!$A$1:$V$2</definedName>
   </definedNames>
-  <calcPr calcId="145621" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
   <pivotCaches>
-    <pivotCache xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cacheId="4" r:id="rId4"/>
+    <pivotCache xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cacheId="16" r:id="rId5"/>
+    <pivotCache xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cacheId="11" r:id="rId6"/>
   </pivotCaches>
 </workbook>
 </file>
@@ -24,11 +25,11 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="#,###,##0;\-#,###,##0;&quot;-&quot;"/>
-    <numFmt numFmtId="165" formatCode="dd\-mmm\-yyyy"/>
-    <numFmt numFmtId="166" formatCode="#,###,##0.00;\-#,###,##0.00;&quot;-&quot;"/>
+    <numFmt numFmtId="164" formatCode="dd\-mmm\-yyyy"/>
+    <numFmt numFmtId="165" formatCode="#,###,##0.00;\-#,###,##0.00;&quot;-&quot;"/>
+    <numFmt numFmtId="166" formatCode="#,##0;\-#,##0;&quot;-&quot;"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,17 +48,8 @@
       <color rgb="FF000000"/>
       <sz val="11"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -67,11 +59,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFC2D8ED"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF4B8C8"/>
       </patternFill>
     </fill>
   </fills>
@@ -117,35 +104,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="1" quotePrefix="0" xfId="0"/>
@@ -153,23 +119,32 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="2">
-    <dxf/>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <border outline="0">
         <left style="thin">
@@ -262,6 +237,34 @@
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheDefinition xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" invalid="0" refreshOnLoad="1" enableRefresh="1" missingItemsLimit="0" createdVersion="3" refreshedVersion="4" minRefreshableVersion="3" recordCount="1" r:id="rId1">
   <cacheSource type="worksheet">
+    <worksheetSource ref="A1:D2" sheet="_PivotSrc"/>
+  </cacheSource>
+  <cacheFields count="4">
+    <cacheField name="Dim1" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
+      <sharedItems count="1">
+        <s v="SYNTHETIC"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Dim2" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
+      <sharedItems count="1">
+        <s v="Synthetic placeholder"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Period" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
+      <sharedItems count="1">
+        <s v="Jan-00"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Value" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
+      <sharedItems count="0" containsInteger="1" containsNumber="1" containsSemiMixedTypes="0" containsString="0" minValue="1" maxValue="1"/>
+    </cacheField>
+  </cacheFields>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" invalid="0" refreshOnLoad="1" enableRefresh="1" missingItemsLimit="0" createdVersion="3" refreshedVersion="4" minRefreshableVersion="3" recordCount="1" r:id="rId1">
+  <cacheSource type="worksheet">
     <worksheetSource ref="A1:V2" sheet="Summary"/>
   </cacheSource>
   <cacheFields count="22">
@@ -310,28 +313,28 @@
     <cacheField name="Expected Invoice Number (From MRN)" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
       <sharedItems count="0" containsBlank="1" containsNonDate="0" containsString="0"/>
     </cacheField>
-    <cacheField name="RECEIPT DATE" uniqueList="1" numFmtId="165" sqlType="0" hierarchy="0" level="0" databaseField="1">
+    <cacheField name="RECEIPT DATE" uniqueList="1" numFmtId="164" sqlType="0" hierarchy="0" level="0" databaseField="1">
       <sharedItems count="0" containsDate="1" containsNonDate="0" containsSemiMixedTypes="0" containsString="0" minDate="2000-01-01T00:00:00" maxDate="2000-01-02T00:00:00"/>
     </cacheField>
     <cacheField name="UOM" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
       <sharedItems count="0"/>
     </cacheField>
-    <cacheField name="RECEIPT QUANTITY" uniqueList="1" numFmtId="166" sqlType="0" hierarchy="0" level="0" databaseField="1">
+    <cacheField name="RECEIPT QUANTITY" uniqueList="1" numFmtId="165" sqlType="0" hierarchy="0" level="0" databaseField="1">
       <sharedItems count="0" containsInteger="1" containsNumber="1" containsSemiMixedTypes="0" containsString="0" minValue="1" maxValue="1"/>
     </cacheField>
-    <cacheField name="BASE AMOUNT" uniqueList="1" numFmtId="166" sqlType="0" hierarchy="0" level="0" databaseField="1">
+    <cacheField name="BASE AMOUNT" uniqueList="1" numFmtId="165" sqlType="0" hierarchy="0" level="0" databaseField="1">
       <sharedItems count="0" containsInteger="1" containsNumber="1" containsSemiMixedTypes="0" containsString="0" minValue="1" maxValue="1"/>
     </cacheField>
     <cacheField name="ITEM GST ENABLED FLAG" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
       <sharedItems count="0"/>
     </cacheField>
-    <cacheField name="CGST" uniqueList="1" numFmtId="166" sqlType="0" hierarchy="0" level="0" databaseField="1">
+    <cacheField name="CGST" uniqueList="1" numFmtId="165" sqlType="0" hierarchy="0" level="0" databaseField="1">
       <sharedItems count="0" containsInteger="1" containsNumber="1" containsSemiMixedTypes="0" containsString="0" minValue="0" maxValue="0"/>
     </cacheField>
-    <cacheField name="SGST" uniqueList="1" numFmtId="166" sqlType="0" hierarchy="0" level="0" databaseField="1">
+    <cacheField name="SGST" uniqueList="1" numFmtId="165" sqlType="0" hierarchy="0" level="0" databaseField="1">
       <sharedItems count="0" containsInteger="1" containsNumber="1" containsSemiMixedTypes="0" containsString="0" minValue="0" maxValue="0"/>
     </cacheField>
-    <cacheField name="IGST" uniqueList="1" numFmtId="166" sqlType="0" hierarchy="0" level="0" databaseField="1">
+    <cacheField name="IGST" uniqueList="1" numFmtId="165" sqlType="0" hierarchy="0" level="0" databaseField="1">
       <sharedItems count="0" containsInteger="1" containsNumber="1" containsSemiMixedTypes="0" containsString="0" minValue="0" maxValue="0"/>
     </cacheField>
     <cacheField name="STATUS" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
@@ -342,6 +345,17 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1">
+  <r>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <n v="1"/>
+  </r>
+</pivotCacheRecords>
+</file>
+
+<file path=xl/pivotCache/pivotCacheRecords2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1">
   <r>
     <x v="0"/>
@@ -371,7 +385,90 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="VendorwisePivot" cacheId="4" dataOnRows="0" dataCaption="Values" showError="0" showMissing="1" updatedVersion="4" minRefreshableVersion="3" asteriskTotals="0" showItems="1" editData="0" disableFieldList="0" showCalcMbrs="0" visualTotals="1" showMultipleLabel="1" showDataDropDown="1" showDrill="1" printDrill="0" showMemberPropertyTips="1" showDataTips="1" enableWizard="1" enableDrill="1" enableFieldProperties="1" preserveFormatting="1" useAutoFormatting="1" pageWrap="0" pageOverThenDown="0" subtotalHiddenItems="0" rowGrandTotals="1" colGrandTotals="1" fieldPrintTitles="0" itemPrintTitles="1" mergeItem="0" showDropZones="1" createdVersion="3" indent="0" showEmptyRow="0" showEmptyCol="0" showHeaders="1" compact="1" outline="1" outlineData="1" compactData="1" published="0" gridDropZones="0" immersive="1" multipleFieldFilters="0" chartFormat="0" rowHeaderCaption="Supplier Name" fieldListSortAscending="0" mdxSubqueries="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" r:id="rId1">
+<pivotTableDefinition xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="LocationwisePivot" cacheId="16" dataOnRows="0" dataCaption="Values" showError="0" showMissing="1" updatedVersion="4" minRefreshableVersion="3" asteriskTotals="0" showItems="1" editData="0" disableFieldList="0" showCalcMbrs="0" visualTotals="1" showMultipleLabel="1" showDataDropDown="1" showDrill="1" printDrill="0" showMemberPropertyTips="1" showDataTips="1" enableWizard="1" enableDrill="1" enableFieldProperties="1" preserveFormatting="1" useAutoFormatting="1" pageWrap="0" pageOverThenDown="0" subtotalHiddenItems="0" rowGrandTotals="1" colGrandTotals="1" fieldPrintTitles="0" itemPrintTitles="1" mergeItem="0" showDropZones="1" createdVersion="3" indent="0" showEmptyRow="0" showEmptyCol="0" showHeaders="1" compact="1" outline="1" outlineData="1" compactData="1" published="0" gridDropZones="0" immersive="1" multipleFieldFilters="0" chartFormat="0" fieldListSortAscending="0" mdxSubqueries="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" r:id="rId1">
+  <location ref="A3:C7" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="4">
+    <pivotField axis="axisRow" showDropDowns="1" compact="1" outline="1" subtotalTop="1" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" itemPageCount="10" sortType="descending" defaultSubtotal="1">
+      <items count="2">
+        <item t="data" sd="1" x="0"/>
+        <item t="default" sd="1"/>
+      </items>
+      <autoSortScope>
+        <pivotArea type="normal" dataOnly="0" outline="0" fieldPosition="0">
+          <references count="1">
+            <reference field="4294967294" selected="0">
+              <x v="0"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
+    </pivotField>
+    <pivotField axis="axisRow" showDropDowns="1" compact="1" outline="1" subtotalTop="1" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" itemPageCount="10" sortType="descending" defaultSubtotal="1">
+      <items count="2">
+        <item t="data" sd="1" x="0"/>
+        <item t="default" sd="1"/>
+      </items>
+      <autoSortScope>
+        <pivotArea type="normal" dataOnly="0" outline="0" fieldPosition="0">
+          <references count="1">
+            <reference field="4294967294" selected="0">
+              <x v="0"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
+    </pivotField>
+    <pivotField axis="axisCol" showDropDowns="1" compact="1" outline="1" subtotalTop="1" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" itemPageCount="10" sortType="manual" defaultSubtotal="1">
+      <items count="2">
+        <item t="data" sd="1" x="0"/>
+        <item t="default" sd="1"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" showDropDowns="1" compact="1" outline="1" subtotalTop="1" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" itemPageCount="10" sortType="manual" defaultSubtotal="1"/>
+  </pivotFields>
+  <rowFields count="2">
+    <field x="0"/>
+    <field x="1"/>
+  </rowFields>
+  <rowItems count="3">
+    <i t="data" r="0" i="0">
+      <x v="0"/>
+    </i>
+    <i t="data" r="1" i="0">
+      <x v="0"/>
+    </i>
+    <i t="grand" r="0" i="0">
+      <x v="0"/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="2"/>
+  </colFields>
+  <colItems count="2">
+    <i t="data" r="0" i="0">
+      <x v="0"/>
+    </i>
+    <i t="grand" r="0" i="0">
+      <x v="0"/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count" fld="3" subtotal="sum" showDataAs="normal" baseField="0" baseItem="0" numFmtId="166"/>
+  </dataFields>
+  <formats count="2">
+    <format action="formatting" dxfId="1">
+      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
+    </format>
+    <format action="formatting">
+      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="VendorwisePivot" cacheId="11" dataOnRows="0" dataCaption="Values" showError="0" showMissing="1" updatedVersion="4" minRefreshableVersion="3" asteriskTotals="0" showItems="1" editData="0" disableFieldList="0" showCalcMbrs="0" visualTotals="1" showMultipleLabel="1" showDataDropDown="1" showDrill="1" printDrill="0" showMemberPropertyTips="1" showDataTips="1" enableWizard="1" enableDrill="1" enableFieldProperties="1" preserveFormatting="1" useAutoFormatting="1" pageWrap="0" pageOverThenDown="0" subtotalHiddenItems="0" rowGrandTotals="1" colGrandTotals="1" fieldPrintTitles="0" itemPrintTitles="1" mergeItem="0" showDropZones="1" createdVersion="3" indent="0" showEmptyRow="0" showEmptyCol="0" showHeaders="1" compact="1" outline="1" outlineData="1" compactData="1" published="0" gridDropZones="0" immersive="1" multipleFieldFilters="0" chartFormat="0" rowHeaderCaption="Supplier Name" fieldListSortAscending="0" mdxSubqueries="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" r:id="rId1">
   <location ref="A3:C6" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="22">
     <pivotField axis="axisCol" showDropDowns="1" compact="1" outline="1" subtotalTop="1" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" itemPageCount="10" sortType="manual" defaultSubtotal="1">
@@ -411,14 +508,14 @@
     <pivotField showDropDowns="1" compact="1" outline="1" subtotalTop="1" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" itemPageCount="10" sortType="manual" defaultSubtotal="1"/>
     <pivotField showDropDowns="1" compact="1" outline="1" subtotalTop="1" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" itemPageCount="10" sortType="manual" defaultSubtotal="1"/>
     <pivotField showDropDowns="1" compact="1" outline="1" subtotalTop="1" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" itemPageCount="10" sortType="manual" defaultSubtotal="1"/>
+    <pivotField showDropDowns="1" compact="1" numFmtId="164" outline="1" subtotalTop="1" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" itemPageCount="10" sortType="manual" defaultSubtotal="1"/>
+    <pivotField showDropDowns="1" compact="1" outline="1" subtotalTop="1" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" itemPageCount="10" sortType="manual" defaultSubtotal="1"/>
+    <pivotField showDropDowns="1" compact="1" numFmtId="165" outline="1" subtotalTop="1" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" itemPageCount="10" sortType="manual" defaultSubtotal="1"/>
     <pivotField showDropDowns="1" compact="1" numFmtId="165" outline="1" subtotalTop="1" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" itemPageCount="10" sortType="manual" defaultSubtotal="1"/>
     <pivotField showDropDowns="1" compact="1" outline="1" subtotalTop="1" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" itemPageCount="10" sortType="manual" defaultSubtotal="1"/>
-    <pivotField showDropDowns="1" compact="1" numFmtId="166" outline="1" subtotalTop="1" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" itemPageCount="10" sortType="manual" defaultSubtotal="1"/>
-    <pivotField showDropDowns="1" compact="1" numFmtId="166" outline="1" subtotalTop="1" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" itemPageCount="10" sortType="manual" defaultSubtotal="1"/>
-    <pivotField showDropDowns="1" compact="1" outline="1" subtotalTop="1" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" itemPageCount="10" sortType="manual" defaultSubtotal="1"/>
-    <pivotField showDropDowns="1" compact="1" numFmtId="166" outline="1" subtotalTop="1" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" itemPageCount="10" sortType="manual" defaultSubtotal="1"/>
-    <pivotField showDropDowns="1" compact="1" numFmtId="166" outline="1" subtotalTop="1" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" itemPageCount="10" sortType="manual" defaultSubtotal="1"/>
-    <pivotField showDropDowns="1" compact="1" numFmtId="166" outline="1" subtotalTop="1" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" itemPageCount="10" sortType="manual" defaultSubtotal="1"/>
+    <pivotField showDropDowns="1" compact="1" numFmtId="165" outline="1" subtotalTop="1" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" itemPageCount="10" sortType="manual" defaultSubtotal="1"/>
+    <pivotField showDropDowns="1" compact="1" numFmtId="165" outline="1" subtotalTop="1" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" itemPageCount="10" sortType="manual" defaultSubtotal="1"/>
+    <pivotField showDropDowns="1" compact="1" numFmtId="165" outline="1" subtotalTop="1" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" itemPageCount="10" sortType="manual" defaultSubtotal="1"/>
     <pivotField showDropDowns="1" compact="1" outline="1" subtotalTop="1" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" itemPageCount="10" sortType="manual" defaultSubtotal="1"/>
   </pivotFields>
   <rowFields count="1">
@@ -447,13 +544,13 @@
     <pageField fld="5" hier="-1"/>
   </pageFields>
   <dataFields count="1">
-    <dataField name="Count of Location" fld="4" subtotal="count" showDataAs="normal" baseField="0" baseItem="0" numFmtId="167"/>
+    <dataField name="Count of Location" fld="4" subtotal="count" showDataAs="normal" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="2">
-    <format action="formatting" dxfId="1">
+    <format action="formatting" dxfId="0">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format action="formatting" dxfId="0">
+    <format action="formatting">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -747,82 +844,148 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="FF375623"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="13" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="21.85546875" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="11.140625" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="15.85546875" bestFit="1" customWidth="1" min="4" max="4"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Location</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Accounts Incharge</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Dim1</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Dim2</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Period</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Synthetic placeholder</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
         <is>
           <t>Jan-00</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Grand Total</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>SYNTHETIC</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Synthetic placeholder</t>
-        </is>
-      </c>
-      <c r="C2" s="16" t="n">
+      <c r="D2" t="n">
         <v>1</v>
       </c>
-      <c r="D2" s="17" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>Grand Total</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="n"/>
-      <c r="C3" s="18">
-        <f>SUBTOTAL(9,C2:C2)</f>
-        <v/>
-      </c>
-      <c r="D3" s="18">
-        <f>SUBTOTAL(9,D2:D2)</f>
-        <v/>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A3:C7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="16.28515625" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="11.28515625" bestFit="1" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Column Labels</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Row Labels</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Jan-00</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Grand Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Synthetic placeholder</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Grand Total</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FF1F6DB1"/>
@@ -838,76 +1001,76 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="B1" s="13" t="inlineStr">
+      <c r="B1" s="8" t="inlineStr">
         <is>
           <t>(All)</t>
         </is>
       </c>
-      <c r="C1" s="13" t="n"/>
+      <c r="C1" s="8" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="n"/>
-      <c r="B2" s="13" t="n"/>
-      <c r="C2" s="13" t="n"/>
+      <c r="A2" s="8" t="n"/>
+      <c r="B2" s="8" t="n"/>
+      <c r="C2" s="8" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>Count of Location</t>
         </is>
       </c>
-      <c r="B3" s="12" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>Column Labels</t>
         </is>
       </c>
-      <c r="C3" s="13" t="n"/>
+      <c r="C3" s="8" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Supplier Name</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>Jan-00</t>
         </is>
       </c>
-      <c r="C4" s="13" t="inlineStr">
+      <c r="C4" s="8" t="inlineStr">
         <is>
           <t>Grand Total</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="14" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Open in Excel to refresh</t>
         </is>
       </c>
-      <c r="B5" s="19" t="n">
+      <c r="B5" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="19" t="n">
+      <c r="C5" s="8" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>Grand Total</t>
         </is>
       </c>
-      <c r="B6" s="19" t="n">
+      <c r="B6" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="C6" s="19" t="n">
+      <c r="C6" s="8" t="n">
         <v>1</v>
       </c>
     </row>
@@ -916,7 +1079,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FF1F6DB1"/>
@@ -951,208 +1114,208 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>ACCOUNTING PERIOD</t>
         </is>
       </c>
-      <c r="B1" s="8" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>SUPPLIER NUMBER</t>
         </is>
       </c>
-      <c r="C1" s="8" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>SUPPLIER NAME</t>
         </is>
       </c>
-      <c r="D1" s="8" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>ORGANIZATION NAME</t>
         </is>
       </c>
-      <c r="E1" s="8" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>SUPPLIER SITE</t>
         </is>
       </c>
-      <c r="F1" s="8" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="G1" s="8" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Accounts Incharge</t>
         </is>
       </c>
-      <c r="H1" s="8" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>PO NUMBER</t>
         </is>
       </c>
-      <c r="I1" s="8" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>ITEM CODE</t>
         </is>
       </c>
-      <c r="J1" s="8" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>LINE DESCRIPTION</t>
         </is>
       </c>
-      <c r="K1" s="8" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>GL ACCOUNT</t>
         </is>
       </c>
-      <c r="L1" s="8" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>RECEIPT NUMBER</t>
         </is>
       </c>
-      <c r="M1" s="8" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Expected Invoice Number (From MRN)</t>
         </is>
       </c>
-      <c r="N1" s="8" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>RECEIPT DATE</t>
         </is>
       </c>
-      <c r="O1" s="8" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>UOM</t>
         </is>
       </c>
-      <c r="P1" s="8" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>RECEIPT QUANTITY</t>
         </is>
       </c>
-      <c r="Q1" s="8" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>BASE AMOUNT</t>
         </is>
       </c>
-      <c r="R1" s="8" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>ITEM GST ENABLED FLAG</t>
         </is>
       </c>
-      <c r="S1" s="8" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>CGST</t>
         </is>
       </c>
-      <c r="T1" s="8" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>SGST</t>
         </is>
       </c>
-      <c r="U1" s="8" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>IGST</t>
         </is>
       </c>
-      <c r="V1" s="8" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>STATUS</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="9" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Jan-00</t>
         </is>
       </c>
-      <c r="B2" s="9" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>SYNTHETIC</t>
         </is>
       </c>
-      <c r="C2" s="9" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Open in Excel to refresh</t>
         </is>
       </c>
-      <c r="D2" s="9" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Synthetic placeholder</t>
         </is>
       </c>
-      <c r="E2" s="9" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>SYNTHETIC</t>
         </is>
       </c>
-      <c r="F2" s="9" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>SYNTHETIC</t>
         </is>
       </c>
-      <c r="G2" s="9" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Synthetic placeholder</t>
         </is>
       </c>
-      <c r="H2" s="9" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>SYNTHETIC</t>
         </is>
       </c>
-      <c r="I2" s="9" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>SYNTHETIC</t>
         </is>
       </c>
-      <c r="J2" s="9" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Synthetic pivot template row</t>
         </is>
       </c>
-      <c r="K2" s="9" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>0000</t>
         </is>
       </c>
-      <c r="L2" s="9" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>SYNTHETIC</t>
         </is>
       </c>
-      <c r="M2" s="9" t="n"/>
-      <c r="N2" s="10" t="n">
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="3" t="n">
         <v>36526</v>
       </c>
-      <c r="O2" s="9" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>EA</t>
         </is>
       </c>
-      <c r="P2" s="11" t="n">
+      <c r="P2" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="Q2" s="11" t="n">
+      <c r="Q2" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R2" s="9" t="inlineStr">
+      <c r="R2" s="2" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="S2" s="11" t="n">
+      <c r="S2" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="T2" s="11" t="n">
+      <c r="T2" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="U2" s="11" t="n">
+      <c r="U2" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="V2" s="9" t="n"/>
+      <c r="V2" s="2" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:V2"/>

</xml_diff>